<commit_message>
roadmap: 0.9 scope — companions, statuses, team memory T0–T4 rows, formulas extended; task 198 claimed (rework resumes on wt/t198)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/2026-09-23-melody-roadmap.xlsx
+++ b/docs/2026-09-23-melody-roadmap.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -732,7 +732,7 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Awaiting approval</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done 2026-09-23</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Rework open (first pass merged)</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Planned at M0's gate</t>
+          <t>Planned at 200's gate</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Friends (manager sessions)</t>
+          <t>Companions (manager sessions)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Names and marks, friend view, send_to_session, limits, manager role</t>
+          <t>Harmony, Tempo, Chord: names and marks, companion view, send_to_session, limits, manager role</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Planned (conflicts settled 2026-09-23)</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1639,20 +1639,390 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>The notebook, live</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>~/Melody: charter, soul, memory index, journal, memories/ (OKF v0.2); weekly health check; lifecycle rules; PRD v2; week-of-use script</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>R, S</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G16" s="5">
+        <f>IFERROR(INDEX(Scales!$B$3:$B$6,MATCH(F16,Scales!$A$3:$A$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="I16" s="5">
+        <f>IFERROR(INDEX(Scales!$E$3:$E$6,MATCH(H16,Scales!$D$3:$D$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="7">
+        <f>IFERROR(ROUND(I16/G16,2),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Done 2026-09-23 (week of use pending)</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>claude -p in ~/Melody recalls the five check-in steps; week script fixture 4 · 3 · 1</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Blue cells (Size, Impact) are Claude's estimates, 2026-09-23, from the program plan v2 and task 181's plan; change them from the dropdowns and the points recalculate.</t>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Trustworthy job outcomes</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Job identity, land events, outcome precedence, linked rework, dedup, one-tap verdicts in the work ledger</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G17" s="5">
+        <f>IFERROR(INDEX(Scales!$B$3:$B$6,MATCH(F17,Scales!$A$3:$A$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I17" s="5">
+        <f>IFERROR(INDEX(Scales!$E$3:$E$6,MATCH(H17,Scales!$D$3:$D$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="7">
+        <f>IFERROR(ROUND(I17/G17,2),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Planned at T0's gate</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>T0, M1a</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>pnpm vitest run ledger-outcome; just walk "job verdict"</t>
+        </is>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Team health, Usage, Team Context</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Team health and Usage tabs; then Team Context (rich editor over memories), Reminders, Clean-up, Companions, Routines</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G18" s="5">
+        <f>IFERROR(INDEX(Scales!$B$3:$B$6,MATCH(F18,Scales!$A$3:$A$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I18" s="5">
+        <f>IFERROR(INDEX(Scales!$E$3:$E$6,MATCH(H18,Scales!$D$3:$D$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="7">
+        <f>IFERROR(ROUND(I18/G18,2),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>M1b, M3</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>just walk "team health"</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Lifecycle routines</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Weekly check-in, budgeted nightly tidy-up (DREAMS.md), cap check, journal archive, worktree sweep, backup, reminders</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>R, P</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G19" s="5">
+        <f>IFERROR(INDEX(Scales!$B$3:$B$6,MATCH(F19,Scales!$A$3:$A$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="I19" s="5">
+        <f>IFERROR(INDEX(Scales!$E$3:$E$6,MATCH(H19,Scales!$D$3:$D$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>IFERROR(ROUND(I19/G19,2),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>M1b, T0</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>fixture: journal byte-identical, ≤25% dropped, stops at budget, idle hour makes no call</t>
+        </is>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Companion growth</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Test sets from judged jobs, pass^3 charter gate, DORA-style scorecard, time horizon, autonomy ladder</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>F, R</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="G20" s="5">
+        <f>IFERROR(INDEX(Scales!$B$3:$B$6,MATCH(F20,Scales!$A$3:$A$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I20" s="5">
+        <f>IFERROR(INDEX(Scales!$E$3:$E$6,MATCH(H20,Scales!$D$3:$D$6,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>IFERROR(ROUND(I20/G20,2),"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>M2, T1</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>a regressing fixture proposal shows "scores lower on &lt;task&gt;"; &lt;3 judged jobs → not enough history</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Blue cells (Size, Impact) are Claude's estimates, 2026-09-23, from the program plan v2 and task 181's plan; change them from the dropdowns and the points recalculate. Updated 2026-09-23: 0.9 is the one target; team memory T0–T4 joined (docs/2026-09-23-team-memory-program-plan-v2.md); friends are now companions.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O15"/>
   <dataValidations count="2">
-    <dataValidation sqref="F2:F15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S,M,L,XL"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Med,High,Very high"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1821,7 +2191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1865,15 +2235,15 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A2,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A2,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C2" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A2,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A2,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D2" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A2,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A2,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -1889,15 +2259,15 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A3,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A3,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C3" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A3,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A3,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A3,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A3,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E3" s="11" t="inlineStr"/>
@@ -1909,15 +2279,15 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A4,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A4,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A4,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A4,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A4,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A4,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
@@ -1929,20 +2299,20 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A5,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A5,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A5,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A5,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A5,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A5,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>blocked on the memory PRD's conflicts</t>
+          <t>companions; conflicts settled 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -1953,15 +2323,15 @@
         </is>
       </c>
       <c r="B6" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A6,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A6,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A6,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A6,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A6,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A6,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E6" s="11" t="inlineStr"/>
@@ -1973,15 +2343,15 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A7,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A7,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A7,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A7,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A7,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A7,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E7" s="11" t="inlineStr"/>
@@ -1993,15 +2363,15 @@
         </is>
       </c>
       <c r="B8" s="11">
-        <f>COUNTIFS(Roadmap!$C$2:$C$15,A8,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A8,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$C$2:$C$15,A8,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A8,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>SUMIFS(Roadmap!$I$2:$I$15,Roadmap!$C$2:$C$15,A8,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A8,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -2011,24 +2381,128 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>T0</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A9,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A9,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A9,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>team memory — in 0.9 since 2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B10" s="11">
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A10,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="C10" s="11">
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A10,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="D10" s="11">
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A10,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="E10" s="11" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B11" s="11">
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A11,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="C11" s="11">
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A11,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="D11" s="11">
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A11,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="E11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A12,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A12,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A12,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="E12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>COUNTIFS(Roadmap!$C$2:$C$20,A13,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="C13" s="11">
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$C$2:$C$20,A13,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>SUMIFS(Roadmap!$I$2:$I$20,Roadmap!$C$2:$C$20,A13,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
+        <v/>
+      </c>
+      <c r="E13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B9" s="13">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="13">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13">
-        <f>SUM(D2:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="13" t="n"/>
+      <c r="B14" s="13">
+        <f>SUM(B2:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="13">
+        <f>SUM(C2:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="13">
+        <f>SUM(D2:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2109,31 +2583,31 @@
         </is>
       </c>
       <c r="B2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$E$2:$E$15,"*F*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$E$2:$E$20,"*F*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$E$2:$E$15,"*U*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$E$2:$E$20,"*U*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$E$2:$E$15,"*R*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$E$2:$E$20,"*R*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$E$2:$E$15,"*P*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$E$2:$E$20,"*P*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="F2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$E$2:$E$15,"*S*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$E$2:$E$20,"*S*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="G2" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A2,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A2,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="H2" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$O$2:$O$15,$A2,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$O$2:$O$20,$A2,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -2149,31 +2623,31 @@
         </is>
       </c>
       <c r="B3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$E$2:$E$15,"*F*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$E$2:$E$20,"*F*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$E$2:$E$15,"*U*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$E$2:$E$20,"*U*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$E$2:$E$15,"*R*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$E$2:$E$20,"*R*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$E$2:$E$15,"*P*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$E$2:$E$20,"*P*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="F3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$E$2:$E$15,"*S*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$E$2:$E$20,"*S*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="G3" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A3,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A3,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="H3" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$O$2:$O$15,$A3,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$O$2:$O$20,$A3,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="I3" s="11" t="inlineStr"/>
@@ -2185,31 +2659,31 @@
         </is>
       </c>
       <c r="B4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$E$2:$E$15,"*F*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$E$2:$E$20,"*F*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="C4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$E$2:$E$15,"*U*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$E$2:$E$20,"*U*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$E$2:$E$15,"*R*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$E$2:$E$20,"*R*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$E$2:$E$15,"*P*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$E$2:$E$20,"*P*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$E$2:$E$15,"*S*",Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$E$2:$E$20,"*S*",Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="G4" s="11">
-        <f>COUNTIFS(Roadmap!$O$2:$O$15,$A4,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>COUNTIFS(Roadmap!$O$2:$O$20,$A4,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="H4" s="11">
-        <f>SUMIFS(Roadmap!$G$2:$G$15,Roadmap!$O$2:$O$15,$A4,Roadmap!$A$2:$A$15,"&lt;&gt;181",Roadmap!$A$2:$A$15,"&lt;&gt;196")</f>
+        <f>SUMIFS(Roadmap!$G$2:$G$20,Roadmap!$O$2:$O$20,$A4,Roadmap!$A$2:$A$20,"&lt;&gt;181",Roadmap!$A$2:$A$20,"&lt;&gt;196")</f>
         <v/>
       </c>
       <c r="I4" s="11" t="inlineStr"/>

</xml_diff>